<commit_message>
Fix five labelling defects found by adversarial verification
- TOTAL MONEY OUT was a subtotal: card payments are cash leaving the bank, so
  the true total is -19,828.58, with the expenses/card split shown beneath it.
  The old pair of headline lines was $522.15 short.
- Monthly and Summary used 'Money out' for figures $522.15 apart; Monthly now
  carries Expenses / Sent to card / Total money out, matching Summary.
- excluded[].postedAt fabricated a posting date for rows that never posted.
- Card liability at both year ends is now derived, not asserted.
- Descriptions named wires and wire fees that do not occur in this year.

Adds evidence.py (48/48 statement months, 73/73 id bijection, boundary margin),
97 live Excel formulas with a recalculation test, and test/gate.sh whose every
check is proven able to fail.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/GCALIT-Mercury-FY2025-26.xlsx
+++ b/docs/GCALIT-Mercury-FY2025-26.xlsx
@@ -128,7 +128,7 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Client and network receipts</t>
+          <t xml:space="preserve">Domestic and international client receipts</t>
         </is>
       </c>
       <c r="C5" s="2">
@@ -146,7 +146,7 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACH credits Mercury files as kind 'other'</t>
+          <t xml:space="preserve">YouTube partner payments, EDI receipts and verification micro-deposits</t>
         </is>
       </c>
       <c r="C6" s="2">
@@ -200,12 +200,12 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Outgoing payments and wires</t>
+          <t xml:space="preserve">  Outgoing payments</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Send Money payments, wires and wire fees</t>
+          <t xml:space="preserve">Send Money payments to suppliers and platforms</t>
         </is>
       </c>
       <c r="C11" s="2">
@@ -223,7 +223,7 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACH debits Mercury files as kind 'other'</t>
+          <t xml:space="preserve">Google ad spend collected by direct debit</t>
         </is>
       </c>
       <c r="C12" s="2">
@@ -399,8 +399,9 @@
     <col min="6" max="6" width="18.92" customWidth="1"/>
     <col min="7" max="7" width="18.92" customWidth="1"/>
     <col min="8" max="8" width="18.92" customWidth="1"/>
-    <col min="9" max="9" width="14.86" customWidth="1"/>
-    <col min="10" max="10" width="10.81" customWidth="1"/>
+    <col min="9" max="9" width="18.92" customWidth="1"/>
+    <col min="10" max="10" width="14.86" customWidth="1"/>
+    <col min="11" max="11" width="10.81" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,7 +422,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Money out</t>
+          <t xml:space="preserve">Expenses</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -431,25 +432,30 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Total money out</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Net</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Closing</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Statement</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Check</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Txns</t>
         </is>
@@ -474,21 +480,25 @@
         <v>0.0</v>
       </c>
       <c r="F2" s="2">
-        <f>C2+D2+E2</f>
+        <f>D2+E2</f>
+        <v>-1.08</v>
+      </c>
+      <c r="G2" s="2">
+        <f>C2+F2</f>
         <v>12010.8</v>
       </c>
-      <c r="G2" s="2">
-        <f>B2+F2</f>
+      <c r="H2" s="2">
+        <f>B2+G2</f>
         <v>28996.2</v>
       </c>
-      <c r="H2" s="2">
+      <c r="I2" s="2">
         <v>28996.2</v>
       </c>
-      <c r="I2" s="0" t="str">
-        <f>IF(G2=H2,"MATCH","MISMATCH")</f>
+      <c r="J2" s="0" t="str">
+        <f>IF(H2=I2,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J2" s="2">
+      <c r="K2" s="2">
         <v>5</v>
       </c>
     </row>
@@ -499,7 +509,7 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>G2</f>
+        <f>H2</f>
         <v>28996.2</v>
       </c>
       <c r="C3" s="2">
@@ -512,21 +522,25 @@
         <v>0.0</v>
       </c>
       <c r="F3" s="2">
-        <f>C3+D3+E3</f>
+        <f>D3+E3</f>
         <v>0.0</v>
       </c>
       <c r="G3" s="2">
-        <f>B3+F3</f>
+        <f>C3+F3</f>
+        <v>0.0</v>
+      </c>
+      <c r="H3" s="2">
+        <f>B3+G3</f>
         <v>28996.2</v>
       </c>
-      <c r="H3" s="2">
+      <c r="I3" s="2">
         <v>28996.2</v>
       </c>
-      <c r="I3" s="0" t="str">
-        <f>IF(G3=H3,"MATCH","MISMATCH")</f>
+      <c r="J3" s="0" t="str">
+        <f>IF(H3=I3,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J3" s="2">
+      <c r="K3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -537,7 +551,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>G3</f>
+        <f>H3</f>
         <v>28996.2</v>
       </c>
       <c r="C4" s="2">
@@ -550,21 +564,25 @@
         <v>0.0</v>
       </c>
       <c r="F4" s="2">
-        <f>C4+D4+E4</f>
+        <f>D4+E4</f>
+        <v>-6.44</v>
+      </c>
+      <c r="G4" s="2">
+        <f>C4+F4</f>
         <v>320.56</v>
       </c>
-      <c r="G4" s="2">
-        <f>B4+F4</f>
+      <c r="H4" s="2">
+        <f>B4+G4</f>
         <v>29316.76</v>
       </c>
-      <c r="H4" s="2">
+      <c r="I4" s="2">
         <v>29316.76</v>
       </c>
-      <c r="I4" s="0" t="str">
-        <f>IF(G4=H4,"MATCH","MISMATCH")</f>
+      <c r="J4" s="0" t="str">
+        <f>IF(H4=I4,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J4" s="2">
+      <c r="K4" s="2">
         <v>2</v>
       </c>
     </row>
@@ -575,7 +593,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>G4</f>
+        <f>H4</f>
         <v>29316.76</v>
       </c>
       <c r="C5" s="2">
@@ -588,21 +606,25 @@
         <v>-241.25</v>
       </c>
       <c r="F5" s="2">
-        <f>C5+D5+E5</f>
+        <f>D5+E5</f>
+        <v>-2640.22</v>
+      </c>
+      <c r="G5" s="2">
+        <f>C5+F5</f>
         <v>5841.17</v>
       </c>
-      <c r="G5" s="2">
-        <f>B5+F5</f>
+      <c r="H5" s="2">
+        <f>B5+G5</f>
         <v>35157.93</v>
       </c>
-      <c r="H5" s="2">
+      <c r="I5" s="2">
         <v>35157.93</v>
       </c>
-      <c r="I5" s="0" t="str">
-        <f>IF(G5=H5,"MATCH","MISMATCH")</f>
+      <c r="J5" s="0" t="str">
+        <f>IF(H5=I5,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J5" s="2">
+      <c r="K5" s="2">
         <v>6</v>
       </c>
     </row>
@@ -613,7 +635,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>G5</f>
+        <f>H5</f>
         <v>35157.93</v>
       </c>
       <c r="C6" s="2">
@@ -626,21 +648,25 @@
         <v>0.0</v>
       </c>
       <c r="F6" s="2">
-        <f>C6+D6+E6</f>
+        <f>D6+E6</f>
+        <v>-6600.54</v>
+      </c>
+      <c r="G6" s="2">
+        <f>C6+F6</f>
         <v>-4457.36</v>
       </c>
-      <c r="G6" s="2">
-        <f>B6+F6</f>
+      <c r="H6" s="2">
+        <f>B6+G6</f>
         <v>30700.57</v>
       </c>
-      <c r="H6" s="2">
+      <c r="I6" s="2">
         <v>30700.57</v>
       </c>
-      <c r="I6" s="0" t="str">
-        <f>IF(G6=H6,"MATCH","MISMATCH")</f>
+      <c r="J6" s="0" t="str">
+        <f>IF(H6=I6,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J6" s="2">
+      <c r="K6" s="2">
         <v>4</v>
       </c>
     </row>
@@ -651,7 +677,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>G6</f>
+        <f>H6</f>
         <v>30700.57</v>
       </c>
       <c r="C7" s="2">
@@ -664,21 +690,25 @@
         <v>0.0</v>
       </c>
       <c r="F7" s="2">
-        <f>C7+D7+E7</f>
+        <f>D7+E7</f>
+        <v>-2359.96</v>
+      </c>
+      <c r="G7" s="2">
+        <f>C7+F7</f>
         <v>3548.06</v>
       </c>
-      <c r="G7" s="2">
-        <f>B7+F7</f>
+      <c r="H7" s="2">
+        <f>B7+G7</f>
         <v>34248.63</v>
       </c>
-      <c r="H7" s="2">
+      <c r="I7" s="2">
         <v>34248.63</v>
       </c>
-      <c r="I7" s="0" t="str">
-        <f>IF(G7=H7,"MATCH","MISMATCH")</f>
+      <c r="J7" s="0" t="str">
+        <f>IF(H7=I7,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J7" s="2">
+      <c r="K7" s="2">
         <v>5</v>
       </c>
     </row>
@@ -689,7 +719,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>G7</f>
+        <f>H7</f>
         <v>34248.63</v>
       </c>
       <c r="C8" s="2">
@@ -702,21 +732,25 @@
         <v>0.0</v>
       </c>
       <c r="F8" s="2">
-        <f>C8+D8+E8</f>
+        <f>D8+E8</f>
+        <v>-3774.6</v>
+      </c>
+      <c r="G8" s="2">
+        <f>C8+F8</f>
         <v>-3633.21</v>
       </c>
-      <c r="G8" s="2">
-        <f>B8+F8</f>
+      <c r="H8" s="2">
+        <f>B8+G8</f>
         <v>30615.42</v>
       </c>
-      <c r="H8" s="2">
+      <c r="I8" s="2">
         <v>30615.42</v>
       </c>
-      <c r="I8" s="0" t="str">
-        <f>IF(G8=H8,"MATCH","MISMATCH")</f>
+      <c r="J8" s="0" t="str">
+        <f>IF(H8=I8,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J8" s="2">
+      <c r="K8" s="2">
         <v>2</v>
       </c>
     </row>
@@ -727,7 +761,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>G8</f>
+        <f>H8</f>
         <v>30615.42</v>
       </c>
       <c r="C9" s="2">
@@ -740,21 +774,25 @@
         <v>-80.9</v>
       </c>
       <c r="F9" s="2">
-        <f>C9+D9+E9</f>
+        <f>D9+E9</f>
+        <v>-80.9</v>
+      </c>
+      <c r="G9" s="2">
+        <f>C9+F9</f>
         <v>98.15</v>
       </c>
-      <c r="G9" s="2">
-        <f>B9+F9</f>
+      <c r="H9" s="2">
+        <f>B9+G9</f>
         <v>30713.57</v>
       </c>
-      <c r="H9" s="2">
+      <c r="I9" s="2">
         <v>30713.57</v>
       </c>
-      <c r="I9" s="0" t="str">
-        <f>IF(G9=H9,"MATCH","MISMATCH")</f>
+      <c r="J9" s="0" t="str">
+        <f>IF(H9=I9,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J9" s="2">
+      <c r="K9" s="2">
         <v>3</v>
       </c>
     </row>
@@ -765,7 +803,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <f>G9</f>
+        <f>H9</f>
         <v>30713.57</v>
       </c>
       <c r="C10" s="2">
@@ -778,21 +816,25 @@
         <v>0.0</v>
       </c>
       <c r="F10" s="2">
-        <f>C10+D10+E10</f>
+        <f>D10+E10</f>
+        <v>-93.06</v>
+      </c>
+      <c r="G10" s="2">
+        <f>C10+F10</f>
         <v>1406.94</v>
       </c>
-      <c r="G10" s="2">
-        <f>B10+F10</f>
+      <c r="H10" s="2">
+        <f>B10+G10</f>
         <v>32120.51</v>
       </c>
-      <c r="H10" s="2">
+      <c r="I10" s="2">
         <v>32120.51</v>
       </c>
-      <c r="I10" s="0" t="str">
-        <f>IF(G10=H10,"MATCH","MISMATCH")</f>
+      <c r="J10" s="0" t="str">
+        <f>IF(H10=I10,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J10" s="2">
+      <c r="K10" s="2">
         <v>2</v>
       </c>
     </row>
@@ -803,7 +845,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <f>G10</f>
+        <f>H10</f>
         <v>32120.51</v>
       </c>
       <c r="C11" s="2">
@@ -816,21 +858,25 @@
         <v>-200.0</v>
       </c>
       <c r="F11" s="2">
-        <f>C11+D11+E11</f>
+        <f>D11+E11</f>
+        <v>-1411.28</v>
+      </c>
+      <c r="G11" s="2">
+        <f>C11+F11</f>
         <v>-124.28</v>
       </c>
-      <c r="G11" s="2">
-        <f>B11+F11</f>
+      <c r="H11" s="2">
+        <f>B11+G11</f>
         <v>31996.23</v>
       </c>
-      <c r="H11" s="2">
+      <c r="I11" s="2">
         <v>31996.23</v>
       </c>
-      <c r="I11" s="0" t="str">
-        <f>IF(G11=H11,"MATCH","MISMATCH")</f>
+      <c r="J11" s="0" t="str">
+        <f>IF(H11=I11,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J11" s="2">
+      <c r="K11" s="2">
         <v>4</v>
       </c>
     </row>
@@ -841,7 +887,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>G11</f>
+        <f>H11</f>
         <v>31996.23</v>
       </c>
       <c r="C12" s="2">
@@ -854,21 +900,25 @@
         <v>0.0</v>
       </c>
       <c r="F12" s="2">
-        <f>C12+D12+E12</f>
+        <f>D12+E12</f>
+        <v>-2000.93</v>
+      </c>
+      <c r="G12" s="2">
+        <f>C12+F12</f>
         <v>-715.78</v>
       </c>
-      <c r="G12" s="2">
-        <f>B12+F12</f>
+      <c r="H12" s="2">
+        <f>B12+G12</f>
         <v>31280.45</v>
       </c>
-      <c r="H12" s="2">
+      <c r="I12" s="2">
         <v>31280.45</v>
       </c>
-      <c r="I12" s="0" t="str">
-        <f>IF(G12=H12,"MATCH","MISMATCH")</f>
+      <c r="J12" s="0" t="str">
+        <f>IF(H12=I12,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J12" s="2">
+      <c r="K12" s="2">
         <v>4</v>
       </c>
     </row>
@@ -879,7 +929,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <f>G12</f>
+        <f>H12</f>
         <v>31280.45</v>
       </c>
       <c r="C13" s="2">
@@ -892,21 +942,25 @@
         <v>0.0</v>
       </c>
       <c r="F13" s="2">
-        <f>C13+D13+E13</f>
+        <f>D13+E13</f>
         <v>-859.57</v>
       </c>
       <c r="G13" s="2">
-        <f>B13+F13</f>
+        <f>C13+F13</f>
+        <v>-859.57</v>
+      </c>
+      <c r="H13" s="2">
+        <f>B13+G13</f>
         <v>30420.88</v>
       </c>
-      <c r="H13" s="2">
+      <c r="I13" s="2">
         <v>30420.88</v>
       </c>
-      <c r="I13" s="0" t="str">
-        <f>IF(G13=H13,"MATCH","MISMATCH")</f>
+      <c r="J13" s="0" t="str">
+        <f>IF(H13=I13,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
-      <c r="J13" s="2">
+      <c r="K13" s="2">
         <v>1</v>
       </c>
     </row>
@@ -934,22 +988,26 @@
       </c>
       <c r="F14" s="3">
         <f>SUM(F2:F13)</f>
+        <v>-19828.58</v>
+      </c>
+      <c r="G14" s="3">
+        <f>C14+F14</f>
         <v>13435.48</v>
       </c>
-      <c r="G14" s="3">
-        <f>B14+F14</f>
+      <c r="H14" s="3">
+        <f>B14+G14</f>
         <v>30420.88</v>
       </c>
-      <c r="H14" s="3">
+      <c r="I14" s="3">
         <v>30420.88</v>
       </c>
-      <c r="I14" s="1" t="inlineStr">
+      <c r="J14" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">MATCH</t>
         </is>
       </c>
-      <c r="J14" s="3">
-        <f>SUM(J2:J13)</f>
+      <c r="K14" s="3">
+        <f>SUM(K2:K13)</f>
         <v>38</v>
       </c>
     </row>
@@ -2808,6 +2866,37 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Card liability 1 Apr 2025</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Credit account opened 2025-05-11, after the year began, and no card charge posted before that</t>
+        </is>
+      </c>
+      <c r="E18" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Card liability 31 Mar 2026</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every charge in the year was paid off or refunded, so the cash and accrual views agree this year</t>
+        </is>
+      </c>
+      <c r="E19" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -2946,7 +3035,7 @@
         </is>
       </c>
       <c r="C5" s="2">
-        <f>Summary!D2+SUM(Ledger!G2:G48)</f>
+        <f>Summary!D2+SUMIF(Ledger!B2:B48,"&lt;&gt;Credit card",Ledger!G2:G48)</f>
         <v>30420.88</v>
       </c>
       <c r="D5" s="2">

</xml_diff>